<commit_message>
Import R results: Australian GP (round 5)
</commit_message>
<xml_diff>
--- a/F1_Standings.xlsx
+++ b/F1_Standings.xlsx
@@ -60892,11 +60892,59 @@
       </c>
     </row>
     <row r="1780" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1780" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1780" t="s">
-        <v>37</v>
+      <c r="A1780" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1780" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1780" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1780">
+        <v>5</v>
+      </c>
+      <c r="E1780" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1780" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1780" t="inlineStr">
+        <is>
+          <t>TomasRodri21</t>
+        </is>
+      </c>
+      <c r="H1780" t="inlineStr">
+        <is>
+          <t>McLaren</t>
+        </is>
+      </c>
+      <c r="I1780">
+        <v>1</v>
+      </c>
+      <c r="J1780">
+        <v>25</v>
+      </c>
+      <c r="K1780" t="inlineStr">
+        <is>
+          <t>83:34.419</t>
+        </is>
+      </c>
+      <c r="L1780" t="inlineStr">
+        <is>
+          <t>1:22.018</t>
+        </is>
       </c>
       <c r="O1780" t="s">
         <v>35</v>
@@ -60906,11 +60954,59 @@
       </c>
     </row>
     <row r="1781" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1781" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1781" t="s">
-        <v>37</v>
+      <c r="A1781" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1781" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1781" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1781">
+        <v>5</v>
+      </c>
+      <c r="E1781" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1781" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1781" t="inlineStr">
+        <is>
+          <t>Charles Leclerc</t>
+        </is>
+      </c>
+      <c r="H1781" t="inlineStr">
+        <is>
+          <t>Ferrari</t>
+        </is>
+      </c>
+      <c r="I1781">
+        <v>2</v>
+      </c>
+      <c r="J1781">
+        <v>18</v>
+      </c>
+      <c r="K1781" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1781" t="inlineStr">
+        <is>
+          <t>1:24.710</t>
+        </is>
       </c>
       <c r="O1781" t="s">
         <v>6</v>
@@ -60920,11 +61016,59 @@
       </c>
     </row>
     <row r="1782" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1782" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1782" t="s">
-        <v>37</v>
+      <c r="A1782" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1782" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1782" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1782">
+        <v>5</v>
+      </c>
+      <c r="E1782" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1782" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1782" t="inlineStr">
+        <is>
+          <t>Kimi Antonelli</t>
+        </is>
+      </c>
+      <c r="H1782" t="inlineStr">
+        <is>
+          <t>Mercedes</t>
+        </is>
+      </c>
+      <c r="I1782">
+        <v>3</v>
+      </c>
+      <c r="J1782">
+        <v>15</v>
+      </c>
+      <c r="K1782" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1782" t="inlineStr">
+        <is>
+          <t>1:24.875</t>
+        </is>
       </c>
       <c r="O1782" t="s">
         <v>10</v>
@@ -60934,11 +61078,59 @@
       </c>
     </row>
     <row r="1783" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1783" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1783" t="s">
-        <v>37</v>
+      <c r="A1783" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1783" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1783" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1783">
+        <v>5</v>
+      </c>
+      <c r="E1783" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1783" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1783" t="inlineStr">
+        <is>
+          <t>Lando Norris</t>
+        </is>
+      </c>
+      <c r="H1783" t="inlineStr">
+        <is>
+          <t>McLaren</t>
+        </is>
+      </c>
+      <c r="I1783">
+        <v>4</v>
+      </c>
+      <c r="J1783">
+        <v>12</v>
+      </c>
+      <c r="K1783" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1783" t="inlineStr">
+        <is>
+          <t>1:25.579</t>
+        </is>
       </c>
       <c r="O1783" t="s">
         <v>79</v>
@@ -60948,11 +61140,59 @@
       </c>
     </row>
     <row r="1784" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1784" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1784" t="s">
-        <v>37</v>
+      <c r="A1784" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1784" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1784" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1784">
+        <v>5</v>
+      </c>
+      <c r="E1784" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1784" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1784" t="inlineStr">
+        <is>
+          <t>Lewis Hamilton</t>
+        </is>
+      </c>
+      <c r="H1784" t="inlineStr">
+        <is>
+          <t>Ferrari</t>
+        </is>
+      </c>
+      <c r="I1784">
+        <v>5</v>
+      </c>
+      <c r="J1784">
+        <v>10</v>
+      </c>
+      <c r="K1784" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1784" t="inlineStr">
+        <is>
+          <t>1:25.103</t>
+        </is>
       </c>
       <c r="O1784" t="s">
         <v>55</v>
@@ -60962,11 +61202,59 @@
       </c>
     </row>
     <row r="1785" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1785" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1785" t="s">
-        <v>37</v>
+      <c r="A1785" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1785" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1785" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1785">
+        <v>5</v>
+      </c>
+      <c r="E1785" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1785" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1785" t="inlineStr">
+        <is>
+          <t>Alexander Albon</t>
+        </is>
+      </c>
+      <c r="H1785" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="I1785">
+        <v>6</v>
+      </c>
+      <c r="J1785">
+        <v>8</v>
+      </c>
+      <c r="K1785" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1785" t="inlineStr">
+        <is>
+          <t>1:25.726</t>
+        </is>
       </c>
       <c r="O1785" t="s">
         <v>11</v>
@@ -60976,131 +61264,899 @@
       </c>
     </row>
     <row r="1786" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1786" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1786" t="s">
-        <v>37</v>
+      <c r="A1786" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1786" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1786" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1786">
+        <v>5</v>
+      </c>
+      <c r="E1786" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1786" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1786" t="inlineStr">
+        <is>
+          <t>Carlos Sainz Jr.</t>
+        </is>
+      </c>
+      <c r="H1786" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="I1786">
+        <v>7</v>
+      </c>
+      <c r="J1786">
+        <v>6</v>
+      </c>
+      <c r="K1786" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1786" t="inlineStr">
+        <is>
+          <t>1:26.150</t>
+        </is>
       </c>
     </row>
     <row r="1787" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1787" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1787" t="s">
-        <v>37</v>
+      <c r="A1787" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1787" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1787" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1787">
+        <v>5</v>
+      </c>
+      <c r="E1787" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1787" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1787" t="inlineStr">
+        <is>
+          <t>Pierre Gasly</t>
+        </is>
+      </c>
+      <c r="H1787" t="inlineStr">
+        <is>
+          <t>Alpine</t>
+        </is>
+      </c>
+      <c r="I1787">
+        <v>8</v>
+      </c>
+      <c r="J1787">
+        <v>4</v>
+      </c>
+      <c r="K1787" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1787" t="inlineStr">
+        <is>
+          <t>1:26.089</t>
+        </is>
       </c>
     </row>
     <row r="1788" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1788" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1788" t="s">
-        <v>37</v>
+      <c r="A1788" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1788" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1788" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1788">
+        <v>5</v>
+      </c>
+      <c r="E1788" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1788" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1788" t="inlineStr">
+        <is>
+          <t>Fernando Alonso</t>
+        </is>
+      </c>
+      <c r="H1788" t="inlineStr">
+        <is>
+          <t>Aston Martin</t>
+        </is>
+      </c>
+      <c r="I1788">
+        <v>9</v>
+      </c>
+      <c r="J1788">
+        <v>2</v>
+      </c>
+      <c r="K1788" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1788" t="inlineStr">
+        <is>
+          <t>1:26.614</t>
+        </is>
       </c>
     </row>
     <row r="1789" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1789" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1789" t="s">
-        <v>37</v>
+      <c r="A1789" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1789" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1789" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1789">
+        <v>5</v>
+      </c>
+      <c r="E1789" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1789" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1789" t="inlineStr">
+        <is>
+          <t>Nico Hülkenberg</t>
+        </is>
+      </c>
+      <c r="H1789" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="I1789">
+        <v>10</v>
+      </c>
+      <c r="J1789">
+        <v>1</v>
+      </c>
+      <c r="K1789" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1789" t="inlineStr">
+        <is>
+          <t>1:26.857</t>
+        </is>
       </c>
     </row>
     <row r="1790" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1790" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1790" t="s">
-        <v>37</v>
+      <c r="A1790" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1790" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1790" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1790">
+        <v>5</v>
+      </c>
+      <c r="E1790" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1790" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1790" t="inlineStr">
+        <is>
+          <t>Arvid Lidblad</t>
+        </is>
+      </c>
+      <c r="H1790" t="inlineStr">
+        <is>
+          <t>Racing Bulls</t>
+        </is>
+      </c>
+      <c r="I1790">
+        <v>11</v>
+      </c>
+      <c r="J1790">
+        <v>0</v>
+      </c>
+      <c r="K1790" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1790" t="inlineStr">
+        <is>
+          <t>1:26.706</t>
+        </is>
       </c>
     </row>
     <row r="1791" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1791" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1791" t="s">
-        <v>37</v>
+      <c r="A1791" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1791" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1791" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1791">
+        <v>5</v>
+      </c>
+      <c r="E1791" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1791" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1791" t="inlineStr">
+        <is>
+          <t>Oliver Bearman</t>
+        </is>
+      </c>
+      <c r="H1791" t="inlineStr">
+        <is>
+          <t>Haas</t>
+        </is>
+      </c>
+      <c r="I1791">
+        <v>12</v>
+      </c>
+      <c r="J1791">
+        <v>0</v>
+      </c>
+      <c r="K1791" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1791" t="inlineStr">
+        <is>
+          <t>1:26.658</t>
+        </is>
       </c>
     </row>
     <row r="1792" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="F1792" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1792" t="s">
-        <v>37</v>
+      <c r="A1792" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1792" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1792" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1792">
+        <v>5</v>
+      </c>
+      <c r="E1792" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1792" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1792" t="inlineStr">
+        <is>
+          <t>Sergio Perez</t>
+        </is>
+      </c>
+      <c r="H1792" t="inlineStr">
+        <is>
+          <t>Cadillac</t>
+        </is>
+      </c>
+      <c r="I1792">
+        <v>13</v>
+      </c>
+      <c r="J1792">
+        <v>0</v>
+      </c>
+      <c r="K1792" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1792" t="inlineStr">
+        <is>
+          <t>1:25.731</t>
+        </is>
       </c>
     </row>
     <row r="1793" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1793" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1793" t="s">
-        <v>37</v>
+      <c r="A1793" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1793" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1793" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1793">
+        <v>5</v>
+      </c>
+      <c r="E1793" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1793" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1793" t="inlineStr">
+        <is>
+          <t>Esteban Ocon</t>
+        </is>
+      </c>
+      <c r="H1793" t="inlineStr">
+        <is>
+          <t>Haas</t>
+        </is>
+      </c>
+      <c r="I1793">
+        <v>14</v>
+      </c>
+      <c r="J1793">
+        <v>0</v>
+      </c>
+      <c r="K1793" t="inlineStr">
+        <is>
+          <t>+2 Laps</t>
+        </is>
+      </c>
+      <c r="L1793" t="inlineStr">
+        <is>
+          <t>1:25.800</t>
+        </is>
       </c>
     </row>
     <row r="1794" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1794" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1794" t="s">
-        <v>37</v>
+      <c r="A1794" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1794" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1794" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1794">
+        <v>5</v>
+      </c>
+      <c r="E1794" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1794" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1794" t="inlineStr">
+        <is>
+          <t>Valtteri Bottas</t>
+        </is>
+      </c>
+      <c r="H1794" t="inlineStr">
+        <is>
+          <t>Cadillac</t>
+        </is>
+      </c>
+      <c r="I1794">
+        <v>15</v>
+      </c>
+      <c r="J1794">
+        <v>0</v>
+      </c>
+      <c r="K1794" t="inlineStr">
+        <is>
+          <t>+2 Laps</t>
+        </is>
+      </c>
+      <c r="L1794" t="inlineStr">
+        <is>
+          <t>1:26.235</t>
+        </is>
       </c>
     </row>
     <row r="1795" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1795" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1795" t="s">
-        <v>37</v>
+      <c r="A1795" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1795" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1795" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1795">
+        <v>5</v>
+      </c>
+      <c r="E1795" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1795" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1795" t="inlineStr">
+        <is>
+          <t>Franco Colapinto</t>
+        </is>
+      </c>
+      <c r="H1795" t="inlineStr">
+        <is>
+          <t>Alpine</t>
+        </is>
+      </c>
+      <c r="I1795">
+        <v>16</v>
+      </c>
+      <c r="J1795">
+        <v>0</v>
+      </c>
+      <c r="K1795" t="inlineStr">
+        <is>
+          <t>+2 Laps</t>
+        </is>
+      </c>
+      <c r="L1795" t="inlineStr">
+        <is>
+          <t>1:27.023</t>
+        </is>
       </c>
     </row>
     <row r="1796" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1796" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1796" t="s">
-        <v>37</v>
+      <c r="A1796" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1796" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1796" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1796">
+        <v>5</v>
+      </c>
+      <c r="E1796" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1796" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1796" t="inlineStr">
+        <is>
+          <t>Liam Lawson</t>
+        </is>
+      </c>
+      <c r="H1796" t="inlineStr">
+        <is>
+          <t>Racing Bulls</t>
+        </is>
+      </c>
+      <c r="I1796">
+        <v>17</v>
+      </c>
+      <c r="J1796">
+        <v>0</v>
+      </c>
+      <c r="K1796" t="inlineStr">
+        <is>
+          <t>+2 Laps</t>
+        </is>
+      </c>
+      <c r="L1796" t="inlineStr">
+        <is>
+          <t>1:26.206</t>
+        </is>
       </c>
     </row>
     <row r="1797" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1797" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1797" t="s">
-        <v>37</v>
+      <c r="A1797" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1797" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1797" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1797">
+        <v>5</v>
+      </c>
+      <c r="E1797" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1797" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1797" t="inlineStr">
+        <is>
+          <t>Lance Stroll</t>
+        </is>
+      </c>
+      <c r="H1797" t="inlineStr">
+        <is>
+          <t>Aston Martin</t>
+        </is>
+      </c>
+      <c r="I1797">
+        <v>18</v>
+      </c>
+      <c r="J1797">
+        <v>0</v>
+      </c>
+      <c r="K1797" t="inlineStr">
+        <is>
+          <t>+2 Laps</t>
+        </is>
+      </c>
+      <c r="L1797" t="inlineStr">
+        <is>
+          <t>1:27.388</t>
+        </is>
       </c>
     </row>
     <row r="1798" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1798" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1798" t="s">
-        <v>37</v>
+      <c r="A1798" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1798" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1798" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1798">
+        <v>5</v>
+      </c>
+      <c r="E1798" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1798" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1798" t="inlineStr">
+        <is>
+          <t>Fatacuida</t>
+        </is>
+      </c>
+      <c r="H1798" t="inlineStr">
+        <is>
+          <t>Mercedes</t>
+        </is>
+      </c>
+      <c r="I1798">
+        <v>19</v>
+      </c>
+      <c r="J1798">
+        <v>0</v>
+      </c>
+      <c r="K1798" t="inlineStr">
+        <is>
+          <t>+6 Laps</t>
+        </is>
+      </c>
+      <c r="L1798" t="inlineStr">
+        <is>
+          <t>1:22.970</t>
+        </is>
       </c>
     </row>
     <row r="1799" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1799" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1799" t="s">
-        <v>37</v>
+      <c r="A1799" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1799" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1799" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1799">
+        <v>5</v>
+      </c>
+      <c r="E1799" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1799" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1799" t="inlineStr">
+        <is>
+          <t>Gabriel Bortoleto</t>
+        </is>
+      </c>
+      <c r="H1799" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="I1799">
+        <v>20</v>
+      </c>
+      <c r="J1799">
+        <v>0</v>
+      </c>
+      <c r="K1799" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="L1799" t="inlineStr">
+        <is>
+          <t>1:26.621</t>
+        </is>
       </c>
     </row>
     <row r="1800" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1800" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1800" t="s">
-        <v>37</v>
+      <c r="A1800" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1800" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1800" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1800">
+        <v>5</v>
+      </c>
+      <c r="E1800" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1800" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1800" t="inlineStr">
+        <is>
+          <t>Max Verstappen</t>
+        </is>
+      </c>
+      <c r="H1800" t="inlineStr">
+        <is>
+          <t>Red Bull</t>
+        </is>
+      </c>
+      <c r="I1800">
+        <v>21</v>
+      </c>
+      <c r="J1800">
+        <v>0</v>
+      </c>
+      <c r="K1800" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="L1800" t="inlineStr">
+        <is>
+          <t>1:25.731</t>
+        </is>
       </c>
     </row>
     <row r="1801" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1801" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1801" t="s">
-        <v>37</v>
+      <c r="A1801" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1801" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1801" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1801">
+        <v>5</v>
+      </c>
+      <c r="E1801" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1801" t="inlineStr">
+        <is>
+          <t>Australian GP</t>
+        </is>
+      </c>
+      <c r="G1801" t="inlineStr">
+        <is>
+          <t>Polingua</t>
+        </is>
+      </c>
+      <c r="H1801" t="inlineStr">
+        <is>
+          <t>Red Bull</t>
+        </is>
+      </c>
+      <c r="I1801">
+        <v>22</v>
+      </c>
+      <c r="J1801">
+        <v>0</v>
+      </c>
+      <c r="K1801" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="L1801" t="inlineStr">
+        <is>
+          <t>1:35.614</t>
+        </is>
       </c>
     </row>
     <row r="1802" spans="6:10" x14ac:dyDescent="0.45">
@@ -85622,8 +86678,10 @@
         <f t="shared" si="4"/>
         <v>Albert Park Circuit</v>
       </c>
-      <c r="F25" t="s">
-        <v>191</v>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
       </c>
       <c r="G25" s="11">
         <v>0.25</v>

</xml_diff>

<commit_message>
Admin: publish reviewed Excel adjustments
</commit_message>
<xml_diff>
--- a/F1_Standings.xlsx
+++ b/F1_Standings.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dfb38b975c490ec7/Documents/GitHub/f1-game-dashboard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruiro\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="13_ncr:1_{424E60AC-F408-4D54-998B-C422FCFB6C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA6EAF35-995A-4E2B-B925-53ADD6A2FCA1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{165239E0-7DB1-4443-8D6D-AA08C95311DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19062" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19210" uniqueCount="431">
   <si>
     <t>Lewis Hamilton</t>
   </si>
@@ -1282,6 +1282,75 @@
   <si>
     <t>+1:09.705</t>
   </si>
+  <si>
+    <t>83:34.419</t>
+  </si>
+  <si>
+    <t>1:22.018</t>
+  </si>
+  <si>
+    <t>1:24.710</t>
+  </si>
+  <si>
+    <t>1:24.875</t>
+  </si>
+  <si>
+    <t>1:25.579</t>
+  </si>
+  <si>
+    <t>1:25.103</t>
+  </si>
+  <si>
+    <t>1:25.726</t>
+  </si>
+  <si>
+    <t>1:26.150</t>
+  </si>
+  <si>
+    <t>1:26.089</t>
+  </si>
+  <si>
+    <t>1:26.614</t>
+  </si>
+  <si>
+    <t>1:26.857</t>
+  </si>
+  <si>
+    <t>1:26.706</t>
+  </si>
+  <si>
+    <t>1:26.658</t>
+  </si>
+  <si>
+    <t>1:25.731</t>
+  </si>
+  <si>
+    <t>1:25.800</t>
+  </si>
+  <si>
+    <t>1:26.235</t>
+  </si>
+  <si>
+    <t>1:27.023</t>
+  </si>
+  <si>
+    <t>1:26.206</t>
+  </si>
+  <si>
+    <t>1:27.388</t>
+  </si>
+  <si>
+    <t>+6 Laps</t>
+  </si>
+  <si>
+    <t>1:22.970</t>
+  </si>
+  <si>
+    <t>1:26.621</t>
+  </si>
+  <si>
+    <t>1:35.614</t>
+  </si>
 </sst>
 </file>
 
@@ -60892,43 +60961,29 @@
       </c>
     </row>
     <row r="1780" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1780" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1780" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1780" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1780" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1780" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1780" t="s">
+        <v>205</v>
       </c>
       <c r="D1780">
         <v>5</v>
       </c>
-      <c r="E1780" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1780" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1780" t="inlineStr">
-        <is>
-          <t>TomasRodri21</t>
-        </is>
-      </c>
-      <c r="H1780" t="inlineStr">
-        <is>
-          <t>McLaren</t>
-        </is>
+      <c r="E1780" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1780" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1780" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1780" t="s">
+        <v>143</v>
       </c>
       <c r="I1780">
         <v>1</v>
@@ -60936,15 +60991,11 @@
       <c r="J1780">
         <v>25</v>
       </c>
-      <c r="K1780" t="inlineStr">
-        <is>
-          <t>83:34.419</t>
-        </is>
-      </c>
-      <c r="L1780" t="inlineStr">
-        <is>
-          <t>1:22.018</t>
-        </is>
+      <c r="K1780" t="s">
+        <v>408</v>
+      </c>
+      <c r="L1780" t="s">
+        <v>409</v>
       </c>
       <c r="O1780" t="s">
         <v>35</v>
@@ -60954,43 +61005,29 @@
       </c>
     </row>
     <row r="1781" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1781" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1781" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1781" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1781" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1781" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1781" t="s">
+        <v>205</v>
       </c>
       <c r="D1781">
         <v>5</v>
       </c>
-      <c r="E1781" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1781" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1781" t="inlineStr">
-        <is>
-          <t>Charles Leclerc</t>
-        </is>
-      </c>
-      <c r="H1781" t="inlineStr">
-        <is>
-          <t>Ferrari</t>
-        </is>
+      <c r="E1781" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1781" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1781" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1781" t="s">
+        <v>138</v>
       </c>
       <c r="I1781">
         <v>2</v>
@@ -60998,15 +61035,11 @@
       <c r="J1781">
         <v>18</v>
       </c>
-      <c r="K1781" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1781" t="inlineStr">
-        <is>
-          <t>1:24.710</t>
-        </is>
+      <c r="K1781" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1781" t="s">
+        <v>410</v>
       </c>
       <c r="O1781" t="s">
         <v>6</v>
@@ -61016,43 +61049,29 @@
       </c>
     </row>
     <row r="1782" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1782" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1782" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1782" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1782" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1782" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1782" t="s">
+        <v>205</v>
       </c>
       <c r="D1782">
         <v>5</v>
       </c>
-      <c r="E1782" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1782" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1782" t="inlineStr">
-        <is>
-          <t>Kimi Antonelli</t>
-        </is>
-      </c>
-      <c r="H1782" t="inlineStr">
-        <is>
-          <t>Mercedes</t>
-        </is>
+      <c r="E1782" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1782" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1782" t="s">
+        <v>200</v>
+      </c>
+      <c r="H1782" t="s">
+        <v>134</v>
       </c>
       <c r="I1782">
         <v>3</v>
@@ -61060,15 +61079,11 @@
       <c r="J1782">
         <v>15</v>
       </c>
-      <c r="K1782" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1782" t="inlineStr">
-        <is>
-          <t>1:24.875</t>
-        </is>
+      <c r="K1782" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1782" t="s">
+        <v>411</v>
       </c>
       <c r="O1782" t="s">
         <v>10</v>
@@ -61078,43 +61093,29 @@
       </c>
     </row>
     <row r="1783" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1783" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1783" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1783" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1783" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1783" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1783" t="s">
+        <v>205</v>
       </c>
       <c r="D1783">
         <v>5</v>
       </c>
-      <c r="E1783" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1783" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1783" t="inlineStr">
-        <is>
-          <t>Lando Norris</t>
-        </is>
-      </c>
-      <c r="H1783" t="inlineStr">
-        <is>
-          <t>McLaren</t>
-        </is>
+      <c r="E1783" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1783" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1783" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1783" t="s">
+        <v>143</v>
       </c>
       <c r="I1783">
         <v>4</v>
@@ -61122,15 +61123,11 @@
       <c r="J1783">
         <v>12</v>
       </c>
-      <c r="K1783" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1783" t="inlineStr">
-        <is>
-          <t>1:25.579</t>
-        </is>
+      <c r="K1783" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1783" t="s">
+        <v>412</v>
       </c>
       <c r="O1783" t="s">
         <v>79</v>
@@ -61140,43 +61137,29 @@
       </c>
     </row>
     <row r="1784" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1784" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1784" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1784" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1784" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1784" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1784" t="s">
+        <v>205</v>
       </c>
       <c r="D1784">
         <v>5</v>
       </c>
-      <c r="E1784" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1784" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1784" t="inlineStr">
-        <is>
-          <t>Lewis Hamilton</t>
-        </is>
-      </c>
-      <c r="H1784" t="inlineStr">
-        <is>
-          <t>Ferrari</t>
-        </is>
+      <c r="E1784" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1784" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1784" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1784" t="s">
+        <v>138</v>
       </c>
       <c r="I1784">
         <v>5</v>
@@ -61184,15 +61167,11 @@
       <c r="J1784">
         <v>10</v>
       </c>
-      <c r="K1784" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1784" t="inlineStr">
-        <is>
-          <t>1:25.103</t>
-        </is>
+      <c r="K1784" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1784" t="s">
+        <v>413</v>
       </c>
       <c r="O1784" t="s">
         <v>55</v>
@@ -61202,43 +61181,29 @@
       </c>
     </row>
     <row r="1785" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1785" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1785" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1785" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1785" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1785" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1785" t="s">
+        <v>205</v>
       </c>
       <c r="D1785">
         <v>5</v>
       </c>
-      <c r="E1785" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1785" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1785" t="inlineStr">
-        <is>
-          <t>Alexander Albon</t>
-        </is>
-      </c>
-      <c r="H1785" t="inlineStr">
-        <is>
-          <t>Williams</t>
-        </is>
+      <c r="E1785" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1785" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1785" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1785" t="s">
+        <v>139</v>
       </c>
       <c r="I1785">
         <v>6</v>
@@ -61246,15 +61211,11 @@
       <c r="J1785">
         <v>8</v>
       </c>
-      <c r="K1785" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1785" t="inlineStr">
-        <is>
-          <t>1:25.726</t>
-        </is>
+      <c r="K1785" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1785" t="s">
+        <v>414</v>
       </c>
       <c r="O1785" t="s">
         <v>11</v>
@@ -61264,43 +61225,29 @@
       </c>
     </row>
     <row r="1786" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1786" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1786" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1786" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1786" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1786" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1786" t="s">
+        <v>205</v>
       </c>
       <c r="D1786">
         <v>5</v>
       </c>
-      <c r="E1786" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1786" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1786" t="inlineStr">
-        <is>
-          <t>Carlos Sainz Jr.</t>
-        </is>
-      </c>
-      <c r="H1786" t="inlineStr">
-        <is>
-          <t>Williams</t>
-        </is>
+      <c r="E1786" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1786" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1786" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1786" t="s">
+        <v>139</v>
       </c>
       <c r="I1786">
         <v>7</v>
@@ -61308,55 +61255,37 @@
       <c r="J1786">
         <v>6</v>
       </c>
-      <c r="K1786" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1786" t="inlineStr">
-        <is>
-          <t>1:26.150</t>
-        </is>
+      <c r="K1786" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1786" t="s">
+        <v>415</v>
       </c>
     </row>
     <row r="1787" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1787" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1787" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1787" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1787" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1787" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1787" t="s">
+        <v>205</v>
       </c>
       <c r="D1787">
         <v>5</v>
       </c>
-      <c r="E1787" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1787" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1787" t="inlineStr">
-        <is>
-          <t>Pierre Gasly</t>
-        </is>
-      </c>
-      <c r="H1787" t="inlineStr">
-        <is>
-          <t>Alpine</t>
-        </is>
+      <c r="E1787" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1787" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1787" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1787" t="s">
+        <v>140</v>
       </c>
       <c r="I1787">
         <v>8</v>
@@ -61364,55 +61293,37 @@
       <c r="J1787">
         <v>4</v>
       </c>
-      <c r="K1787" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1787" t="inlineStr">
-        <is>
-          <t>1:26.089</t>
-        </is>
+      <c r="K1787" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1787" t="s">
+        <v>416</v>
       </c>
     </row>
     <row r="1788" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1788" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1788" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1788" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1788" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1788" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1788" t="s">
+        <v>205</v>
       </c>
       <c r="D1788">
         <v>5</v>
       </c>
-      <c r="E1788" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1788" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1788" t="inlineStr">
-        <is>
-          <t>Fernando Alonso</t>
-        </is>
-      </c>
-      <c r="H1788" t="inlineStr">
-        <is>
-          <t>Aston Martin</t>
-        </is>
+      <c r="E1788" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1788" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1788" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1788" t="s">
+        <v>133</v>
       </c>
       <c r="I1788">
         <v>9</v>
@@ -61420,55 +61331,37 @@
       <c r="J1788">
         <v>2</v>
       </c>
-      <c r="K1788" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1788" t="inlineStr">
-        <is>
-          <t>1:26.614</t>
-        </is>
+      <c r="K1788" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1788" t="s">
+        <v>417</v>
       </c>
     </row>
     <row r="1789" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1789" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1789" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1789" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1789" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1789" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1789" t="s">
+        <v>205</v>
       </c>
       <c r="D1789">
         <v>5</v>
       </c>
-      <c r="E1789" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1789" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1789" t="inlineStr">
-        <is>
-          <t>Nico Hülkenberg</t>
-        </is>
-      </c>
-      <c r="H1789" t="inlineStr">
-        <is>
-          <t>Audi</t>
-        </is>
+      <c r="E1789" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1789" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1789" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1789" t="s">
+        <v>198</v>
       </c>
       <c r="I1789">
         <v>10</v>
@@ -61476,55 +61369,37 @@
       <c r="J1789">
         <v>1</v>
       </c>
-      <c r="K1789" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1789" t="inlineStr">
-        <is>
-          <t>1:26.857</t>
-        </is>
+      <c r="K1789" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1789" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="1790" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1790" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1790" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1790" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1790" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1790" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1790" t="s">
+        <v>205</v>
       </c>
       <c r="D1790">
         <v>5</v>
       </c>
-      <c r="E1790" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1790" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1790" t="inlineStr">
-        <is>
-          <t>Arvid Lidblad</t>
-        </is>
-      </c>
-      <c r="H1790" t="inlineStr">
-        <is>
-          <t>Racing Bulls</t>
-        </is>
+      <c r="E1790" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1790" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1790" t="s">
+        <v>202</v>
+      </c>
+      <c r="H1790" t="s">
+        <v>144</v>
       </c>
       <c r="I1790">
         <v>11</v>
@@ -61532,55 +61407,37 @@
       <c r="J1790">
         <v>0</v>
       </c>
-      <c r="K1790" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1790" t="inlineStr">
-        <is>
-          <t>1:26.706</t>
-        </is>
+      <c r="K1790" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1790" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="1791" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1791" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1791" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1791" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1791" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1791" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1791" t="s">
+        <v>205</v>
       </c>
       <c r="D1791">
         <v>5</v>
       </c>
-      <c r="E1791" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1791" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1791" t="inlineStr">
-        <is>
-          <t>Oliver Bearman</t>
-        </is>
-      </c>
-      <c r="H1791" t="inlineStr">
-        <is>
-          <t>Haas</t>
-        </is>
+      <c r="E1791" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1791" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1791" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1791" t="s">
+        <v>137</v>
       </c>
       <c r="I1791">
         <v>12</v>
@@ -61588,55 +61445,37 @@
       <c r="J1791">
         <v>0</v>
       </c>
-      <c r="K1791" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1791" t="inlineStr">
-        <is>
-          <t>1:26.658</t>
-        </is>
+      <c r="K1791" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1791" t="s">
+        <v>420</v>
       </c>
     </row>
     <row r="1792" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1792" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1792" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1792" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="A1792" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1792" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1792" t="s">
+        <v>205</v>
       </c>
       <c r="D1792">
         <v>5</v>
       </c>
-      <c r="E1792" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1792" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1792" t="inlineStr">
-        <is>
-          <t>Sergio Perez</t>
-        </is>
-      </c>
-      <c r="H1792" t="inlineStr">
-        <is>
-          <t>Cadillac</t>
-        </is>
+      <c r="E1792" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1792" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1792" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1792" t="s">
+        <v>199</v>
       </c>
       <c r="I1792">
         <v>13</v>
@@ -61644,55 +61483,37 @@
       <c r="J1792">
         <v>0</v>
       </c>
-      <c r="K1792" t="inlineStr">
-        <is>
-          <t>+1 Lap</t>
-        </is>
-      </c>
-      <c r="L1792" t="inlineStr">
-        <is>
-          <t>1:25.731</t>
-        </is>
-      </c>
-    </row>
-    <row r="1793" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="A1793" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1793" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1793" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="K1792" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1792" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="1793" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1793" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1793" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1793" t="s">
+        <v>205</v>
       </c>
       <c r="D1793">
         <v>5</v>
       </c>
-      <c r="E1793" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1793" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1793" t="inlineStr">
-        <is>
-          <t>Esteban Ocon</t>
-        </is>
-      </c>
-      <c r="H1793" t="inlineStr">
-        <is>
-          <t>Haas</t>
-        </is>
+      <c r="E1793" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1793" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1793" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1793" t="s">
+        <v>137</v>
       </c>
       <c r="I1793">
         <v>14</v>
@@ -61700,55 +61521,37 @@
       <c r="J1793">
         <v>0</v>
       </c>
-      <c r="K1793" t="inlineStr">
-        <is>
-          <t>+2 Laps</t>
-        </is>
-      </c>
-      <c r="L1793" t="inlineStr">
-        <is>
-          <t>1:25.800</t>
-        </is>
-      </c>
-    </row>
-    <row r="1794" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="A1794" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1794" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1794" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="K1793" t="s">
+        <v>238</v>
+      </c>
+      <c r="L1793" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="1794" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1794" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1794" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1794" t="s">
+        <v>205</v>
       </c>
       <c r="D1794">
         <v>5</v>
       </c>
-      <c r="E1794" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1794" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1794" t="inlineStr">
-        <is>
-          <t>Valtteri Bottas</t>
-        </is>
-      </c>
-      <c r="H1794" t="inlineStr">
-        <is>
-          <t>Cadillac</t>
-        </is>
+      <c r="E1794" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1794" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1794" t="s">
+        <v>79</v>
+      </c>
+      <c r="H1794" t="s">
+        <v>199</v>
       </c>
       <c r="I1794">
         <v>15</v>
@@ -61756,55 +61559,37 @@
       <c r="J1794">
         <v>0</v>
       </c>
-      <c r="K1794" t="inlineStr">
-        <is>
-          <t>+2 Laps</t>
-        </is>
-      </c>
-      <c r="L1794" t="inlineStr">
-        <is>
-          <t>1:26.235</t>
-        </is>
-      </c>
-    </row>
-    <row r="1795" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="A1795" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1795" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1795" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="K1794" t="s">
+        <v>238</v>
+      </c>
+      <c r="L1794" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="1795" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1795" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1795" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1795" t="s">
+        <v>205</v>
       </c>
       <c r="D1795">
         <v>5</v>
       </c>
-      <c r="E1795" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1795" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1795" t="inlineStr">
-        <is>
-          <t>Franco Colapinto</t>
-        </is>
-      </c>
-      <c r="H1795" t="inlineStr">
-        <is>
-          <t>Alpine</t>
-        </is>
+      <c r="E1795" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1795" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1795" t="s">
+        <v>201</v>
+      </c>
+      <c r="H1795" t="s">
+        <v>140</v>
       </c>
       <c r="I1795">
         <v>16</v>
@@ -61812,55 +61597,37 @@
       <c r="J1795">
         <v>0</v>
       </c>
-      <c r="K1795" t="inlineStr">
-        <is>
-          <t>+2 Laps</t>
-        </is>
-      </c>
-      <c r="L1795" t="inlineStr">
-        <is>
-          <t>1:27.023</t>
-        </is>
-      </c>
-    </row>
-    <row r="1796" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="A1796" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1796" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1796" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="K1795" t="s">
+        <v>238</v>
+      </c>
+      <c r="L1795" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="1796" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1796" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1796" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1796" t="s">
+        <v>205</v>
       </c>
       <c r="D1796">
         <v>5</v>
       </c>
-      <c r="E1796" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1796" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1796" t="inlineStr">
-        <is>
-          <t>Liam Lawson</t>
-        </is>
-      </c>
-      <c r="H1796" t="inlineStr">
-        <is>
-          <t>Racing Bulls</t>
-        </is>
+      <c r="E1796" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1796" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1796" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1796" t="s">
+        <v>144</v>
       </c>
       <c r="I1796">
         <v>17</v>
@@ -61868,55 +61635,37 @@
       <c r="J1796">
         <v>0</v>
       </c>
-      <c r="K1796" t="inlineStr">
-        <is>
-          <t>+2 Laps</t>
-        </is>
-      </c>
-      <c r="L1796" t="inlineStr">
-        <is>
-          <t>1:26.206</t>
-        </is>
-      </c>
-    </row>
-    <row r="1797" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="A1797" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1797" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1797" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="K1796" t="s">
+        <v>238</v>
+      </c>
+      <c r="L1796" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="1797" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1797" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1797" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1797" t="s">
+        <v>205</v>
       </c>
       <c r="D1797">
         <v>5</v>
       </c>
-      <c r="E1797" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1797" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1797" t="inlineStr">
-        <is>
-          <t>Lance Stroll</t>
-        </is>
-      </c>
-      <c r="H1797" t="inlineStr">
-        <is>
-          <t>Aston Martin</t>
-        </is>
+      <c r="E1797" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1797" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1797" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1797" t="s">
+        <v>133</v>
       </c>
       <c r="I1797">
         <v>18</v>
@@ -61924,55 +61673,37 @@
       <c r="J1797">
         <v>0</v>
       </c>
-      <c r="K1797" t="inlineStr">
-        <is>
-          <t>+2 Laps</t>
-        </is>
-      </c>
-      <c r="L1797" t="inlineStr">
-        <is>
-          <t>1:27.388</t>
-        </is>
-      </c>
-    </row>
-    <row r="1798" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="A1798" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1798" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1798" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="K1797" t="s">
+        <v>238</v>
+      </c>
+      <c r="L1797" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="1798" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1798" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1798" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1798" t="s">
+        <v>205</v>
       </c>
       <c r="D1798">
         <v>5</v>
       </c>
-      <c r="E1798" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1798" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1798" t="inlineStr">
-        <is>
-          <t>Fatacuida</t>
-        </is>
-      </c>
-      <c r="H1798" t="inlineStr">
-        <is>
-          <t>Mercedes</t>
-        </is>
+      <c r="E1798" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1798" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1798" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1798" t="s">
+        <v>134</v>
       </c>
       <c r="I1798">
         <v>19</v>
@@ -61980,55 +61711,37 @@
       <c r="J1798">
         <v>0</v>
       </c>
-      <c r="K1798" t="inlineStr">
-        <is>
-          <t>+6 Laps</t>
-        </is>
-      </c>
-      <c r="L1798" t="inlineStr">
-        <is>
-          <t>1:22.970</t>
-        </is>
-      </c>
-    </row>
-    <row r="1799" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="A1799" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1799" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1799" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="K1798" t="s">
+        <v>427</v>
+      </c>
+      <c r="L1798" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="1799" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1799" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1799" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1799" t="s">
+        <v>205</v>
       </c>
       <c r="D1799">
         <v>5</v>
       </c>
-      <c r="E1799" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1799" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1799" t="inlineStr">
-        <is>
-          <t>Gabriel Bortoleto</t>
-        </is>
-      </c>
-      <c r="H1799" t="inlineStr">
-        <is>
-          <t>Audi</t>
-        </is>
+      <c r="E1799" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1799" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1799" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1799" t="s">
+        <v>198</v>
       </c>
       <c r="I1799">
         <v>20</v>
@@ -62036,55 +61749,37 @@
       <c r="J1799">
         <v>0</v>
       </c>
-      <c r="K1799" t="inlineStr">
-        <is>
-          <t>DNF</t>
-        </is>
-      </c>
-      <c r="L1799" t="inlineStr">
-        <is>
-          <t>1:26.621</t>
-        </is>
-      </c>
-    </row>
-    <row r="1800" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="A1800" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1800" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1800" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="K1799" t="s">
+        <v>194</v>
+      </c>
+      <c r="L1799" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="1800" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1800" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1800" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1800" t="s">
+        <v>205</v>
       </c>
       <c r="D1800">
         <v>5</v>
       </c>
-      <c r="E1800" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1800" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1800" t="inlineStr">
-        <is>
-          <t>Max Verstappen</t>
-        </is>
-      </c>
-      <c r="H1800" t="inlineStr">
-        <is>
-          <t>Red Bull</t>
-        </is>
+      <c r="E1800" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1800" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1800" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1800" t="s">
+        <v>135</v>
       </c>
       <c r="I1800">
         <v>21</v>
@@ -62092,55 +61787,37 @@
       <c r="J1800">
         <v>0</v>
       </c>
-      <c r="K1800" t="inlineStr">
-        <is>
-          <t>DNF</t>
-        </is>
-      </c>
-      <c r="L1800" t="inlineStr">
-        <is>
-          <t>1:25.731</t>
-        </is>
-      </c>
-    </row>
-    <row r="1801" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="A1801" t="inlineStr">
-        <is>
-          <t>F1 25: 2026 Season pack</t>
-        </is>
-      </c>
-      <c r="B1801" t="inlineStr">
-        <is>
-          <t>2026-T02</t>
-        </is>
-      </c>
-      <c r="C1801" t="inlineStr">
-        <is>
-          <t>Teikirise</t>
-        </is>
+      <c r="K1800" t="s">
+        <v>194</v>
+      </c>
+      <c r="L1800" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="1801" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1801" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1801" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1801" t="s">
+        <v>205</v>
       </c>
       <c r="D1801">
         <v>5</v>
       </c>
-      <c r="E1801" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F1801" t="inlineStr">
-        <is>
-          <t>Australian GP</t>
-        </is>
-      </c>
-      <c r="G1801" t="inlineStr">
-        <is>
-          <t>Polingua</t>
-        </is>
-      </c>
-      <c r="H1801" t="inlineStr">
-        <is>
-          <t>Red Bull</t>
-        </is>
+      <c r="E1801" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1801" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1801" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1801" t="s">
+        <v>135</v>
       </c>
       <c r="I1801">
         <v>22</v>
@@ -62148,18 +61825,14 @@
       <c r="J1801">
         <v>0</v>
       </c>
-      <c r="K1801" t="inlineStr">
-        <is>
-          <t>DNF</t>
-        </is>
-      </c>
-      <c r="L1801" t="inlineStr">
-        <is>
-          <t>1:35.614</t>
-        </is>
-      </c>
-    </row>
-    <row r="1802" spans="6:10" x14ac:dyDescent="0.45">
+      <c r="K1801" t="s">
+        <v>194</v>
+      </c>
+      <c r="L1801" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="1802" spans="1:12" x14ac:dyDescent="0.45">
       <c r="F1802" t="s">
         <v>37</v>
       </c>
@@ -62167,7 +61840,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="1803" spans="6:10" x14ac:dyDescent="0.45">
+    <row r="1803" spans="1:12" x14ac:dyDescent="0.45">
       <c r="F1803" t="s">
         <v>37</v>
       </c>
@@ -62175,7 +61848,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="1804" spans="6:10" x14ac:dyDescent="0.45">
+    <row r="1804" spans="1:12" x14ac:dyDescent="0.45">
       <c r="F1804" t="s">
         <v>37</v>
       </c>
@@ -62183,7 +61856,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="1805" spans="6:10" x14ac:dyDescent="0.45">
+    <row r="1805" spans="1:12" x14ac:dyDescent="0.45">
       <c r="F1805" t="s">
         <v>37</v>
       </c>
@@ -62191,7 +61864,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="1806" spans="6:10" x14ac:dyDescent="0.45">
+    <row r="1806" spans="1:12" x14ac:dyDescent="0.45">
       <c r="F1806" t="s">
         <v>37</v>
       </c>
@@ -62199,7 +61872,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="1807" spans="6:10" x14ac:dyDescent="0.45">
+    <row r="1807" spans="1:12" x14ac:dyDescent="0.45">
       <c r="F1807" t="s">
         <v>37</v>
       </c>
@@ -62207,7 +61880,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="1808" spans="6:10" x14ac:dyDescent="0.45">
+    <row r="1808" spans="1:12" x14ac:dyDescent="0.45">
       <c r="F1808" t="s">
         <v>37</v>
       </c>
@@ -86678,10 +86351,8 @@
         <f t="shared" si="4"/>
         <v>Albert Park Circuit</v>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
+      <c r="F25" t="s">
+        <v>190</v>
       </c>
       <c r="G25" s="11">
         <v>0.25</v>
@@ -86860,11 +86531,11 @@
         <v>46313</v>
       </c>
       <c r="D31" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="E31" t="str">
-        <f t="shared" si="5"/>
-        <v>Circuit de Barcelona-Catalunya</v>
+        <f t="shared" ref="E31" si="6">VLOOKUP(D31,$K$1:$L$43,2,FALSE)</f>
+        <v>Algarve International Circuit</v>
       </c>
       <c r="F31" t="s">
         <v>191</v>
@@ -87159,11 +86830,11 @@
         <v>46390</v>
       </c>
       <c r="D42" t="s">
-        <v>121</v>
+        <v>20</v>
       </c>
       <c r="E42" t="str">
-        <f t="shared" si="5"/>
-        <v>Circuit de Monaco</v>
+        <f t="shared" ref="E42" si="7">VLOOKUP(D42,$K$1:$L$43,2,FALSE)</f>
+        <v>Miami International Autodrome</v>
       </c>
       <c r="F42" t="s">
         <v>191</v>
@@ -87173,55 +86844,12 @@
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A43" t="s">
-        <v>205</v>
-      </c>
-      <c r="B43">
-        <f t="shared" si="1"/>
-        <v>23</v>
-      </c>
-      <c r="C43" s="8">
-        <v>46397</v>
-      </c>
-      <c r="D43" t="s">
-        <v>120</v>
-      </c>
-      <c r="E43" t="str">
-        <f t="shared" si="5"/>
-        <v>Algarve International Circuit</v>
-      </c>
-      <c r="F43" t="s">
-        <v>191</v>
-      </c>
-      <c r="G43" s="11">
-        <v>0.25</v>
-      </c>
+      <c r="C43" s="8"/>
+      <c r="G43" s="11"/>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A44" t="s">
-        <v>205</v>
-      </c>
-      <c r="B44">
-        <f t="shared" si="1"/>
-        <v>24</v>
-      </c>
-      <c r="C44" s="8">
-        <f>C43+7</f>
-        <v>46404</v>
-      </c>
-      <c r="D44" t="s">
-        <v>20</v>
-      </c>
-      <c r="E44" t="str">
-        <f t="shared" si="5"/>
-        <v>Miami International Autodrome</v>
-      </c>
-      <c r="F44" t="s">
-        <v>191</v>
-      </c>
-      <c r="G44" s="11">
-        <v>0.25</v>
-      </c>
+      <c r="C44" s="8"/>
+      <c r="G44" s="11"/>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.45">
       <c r="C45" s="8"/>

</xml_diff>

<commit_message>
Rename Barcelona-Catalunya and Spanish GP in Calendar and Leagues
</commit_message>
<xml_diff>
--- a/F1_Standings.xlsx
+++ b/F1_Standings.xlsx
@@ -9696,8 +9696,10 @@
       <c r="E248" t="s">
         <v>207</v>
       </c>
-      <c r="F248" t="s">
-        <v>113</v>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G248" t="s">
         <v>55</v>
@@ -9728,8 +9730,10 @@
       <c r="E249" t="s">
         <v>207</v>
       </c>
-      <c r="F249" t="s">
-        <v>113</v>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G249" t="s">
         <v>68</v>
@@ -9760,8 +9764,10 @@
       <c r="E250" t="s">
         <v>207</v>
       </c>
-      <c r="F250" t="s">
-        <v>113</v>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G250" t="s">
         <v>45</v>
@@ -9792,8 +9798,10 @@
       <c r="E251" t="s">
         <v>207</v>
       </c>
-      <c r="F251" t="s">
-        <v>113</v>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G251" t="s">
         <v>6</v>
@@ -9824,8 +9832,10 @@
       <c r="E252" t="s">
         <v>207</v>
       </c>
-      <c r="F252" t="s">
-        <v>113</v>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G252" t="s">
         <v>2</v>
@@ -9856,8 +9866,10 @@
       <c r="E253" t="s">
         <v>207</v>
       </c>
-      <c r="F253" t="s">
-        <v>113</v>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G253" t="s">
         <v>110</v>
@@ -9888,8 +9900,10 @@
       <c r="E254" t="s">
         <v>207</v>
       </c>
-      <c r="F254" t="s">
-        <v>113</v>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G254" t="s">
         <v>43</v>
@@ -9920,8 +9934,10 @@
       <c r="E255" t="s">
         <v>207</v>
       </c>
-      <c r="F255" t="s">
-        <v>113</v>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G255" t="s">
         <v>5</v>
@@ -9952,8 +9968,10 @@
       <c r="E256" t="s">
         <v>207</v>
       </c>
-      <c r="F256" t="s">
-        <v>113</v>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G256" t="s">
         <v>8</v>
@@ -9984,8 +10002,10 @@
       <c r="E257" t="s">
         <v>207</v>
       </c>
-      <c r="F257" t="s">
-        <v>113</v>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G257" t="s">
         <v>48</v>
@@ -10016,8 +10036,10 @@
       <c r="E258" t="s">
         <v>207</v>
       </c>
-      <c r="F258" t="s">
-        <v>113</v>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G258" t="s">
         <v>70</v>
@@ -10048,8 +10070,10 @@
       <c r="E259" t="s">
         <v>207</v>
       </c>
-      <c r="F259" t="s">
-        <v>113</v>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G259" t="s">
         <v>4</v>
@@ -10080,8 +10104,10 @@
       <c r="E260" t="s">
         <v>207</v>
       </c>
-      <c r="F260" t="s">
-        <v>113</v>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G260" t="s">
         <v>33</v>
@@ -10112,8 +10138,10 @@
       <c r="E261" t="s">
         <v>207</v>
       </c>
-      <c r="F261" t="s">
-        <v>113</v>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G261" t="s">
         <v>34</v>
@@ -10144,8 +10172,10 @@
       <c r="E262" t="s">
         <v>207</v>
       </c>
-      <c r="F262" t="s">
-        <v>113</v>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G262" t="s">
         <v>71</v>
@@ -10176,8 +10206,10 @@
       <c r="E263" t="s">
         <v>207</v>
       </c>
-      <c r="F263" t="s">
-        <v>113</v>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G263" t="s">
         <v>9</v>
@@ -10208,8 +10240,10 @@
       <c r="E264" t="s">
         <v>207</v>
       </c>
-      <c r="F264" t="s">
-        <v>113</v>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G264" t="s">
         <v>69</v>
@@ -10240,8 +10274,10 @@
       <c r="E265" t="s">
         <v>207</v>
       </c>
-      <c r="F265" t="s">
-        <v>113</v>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G265" t="s">
         <v>3</v>
@@ -10272,8 +10308,10 @@
       <c r="E266" t="s">
         <v>207</v>
       </c>
-      <c r="F266" t="s">
-        <v>113</v>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G266" t="s">
         <v>32</v>
@@ -10304,8 +10342,10 @@
       <c r="E267" t="s">
         <v>207</v>
       </c>
-      <c r="F267" t="s">
-        <v>113</v>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G267" t="s">
         <v>11</v>
@@ -34656,8 +34696,10 @@
       <c r="E1028" t="s">
         <v>207</v>
       </c>
-      <c r="F1028" t="s">
-        <v>113</v>
+      <c r="F1028" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1028" t="s">
         <v>1</v>
@@ -34688,8 +34730,10 @@
       <c r="E1029" t="s">
         <v>207</v>
       </c>
-      <c r="F1029" t="s">
-        <v>113</v>
+      <c r="F1029" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1029" t="s">
         <v>7</v>
@@ -34720,8 +34764,10 @@
       <c r="E1030" t="s">
         <v>207</v>
       </c>
-      <c r="F1030" t="s">
-        <v>113</v>
+      <c r="F1030" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1030" t="s">
         <v>85</v>
@@ -34752,8 +34798,10 @@
       <c r="E1031" t="s">
         <v>207</v>
       </c>
-      <c r="F1031" t="s">
-        <v>113</v>
+      <c r="F1031" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1031" t="s">
         <v>32</v>
@@ -34784,8 +34832,10 @@
       <c r="E1032" t="s">
         <v>207</v>
       </c>
-      <c r="F1032" t="s">
-        <v>113</v>
+      <c r="F1032" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1032" t="s">
         <v>0</v>
@@ -34816,8 +34866,10 @@
       <c r="E1033" t="s">
         <v>207</v>
       </c>
-      <c r="F1033" t="s">
-        <v>113</v>
+      <c r="F1033" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1033" t="s">
         <v>6</v>
@@ -34848,8 +34900,10 @@
       <c r="E1034" t="s">
         <v>207</v>
       </c>
-      <c r="F1034" t="s">
-        <v>113</v>
+      <c r="F1034" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1034" t="s">
         <v>2</v>
@@ -34880,8 +34934,10 @@
       <c r="E1035" t="s">
         <v>207</v>
       </c>
-      <c r="F1035" t="s">
-        <v>113</v>
+      <c r="F1035" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1035" t="s">
         <v>4</v>
@@ -34912,8 +34968,10 @@
       <c r="E1036" t="s">
         <v>207</v>
       </c>
-      <c r="F1036" t="s">
-        <v>113</v>
+      <c r="F1036" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1036" t="s">
         <v>3</v>
@@ -34944,8 +35002,10 @@
       <c r="E1037" t="s">
         <v>207</v>
       </c>
-      <c r="F1037" t="s">
-        <v>113</v>
+      <c r="F1037" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1037" t="s">
         <v>68</v>
@@ -34976,8 +35036,10 @@
       <c r="E1038" t="s">
         <v>207</v>
       </c>
-      <c r="F1038" t="s">
-        <v>113</v>
+      <c r="F1038" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1038" t="s">
         <v>36</v>
@@ -35008,8 +35070,10 @@
       <c r="E1039" t="s">
         <v>207</v>
       </c>
-      <c r="F1039" t="s">
-        <v>113</v>
+      <c r="F1039" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1039" t="s">
         <v>86</v>
@@ -35040,8 +35104,10 @@
       <c r="E1040" t="s">
         <v>207</v>
       </c>
-      <c r="F1040" t="s">
-        <v>113</v>
+      <c r="F1040" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1040" t="s">
         <v>5</v>
@@ -35072,8 +35138,10 @@
       <c r="E1041" t="s">
         <v>207</v>
       </c>
-      <c r="F1041" t="s">
-        <v>113</v>
+      <c r="F1041" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1041" t="s">
         <v>9</v>
@@ -35104,8 +35172,10 @@
       <c r="E1042" t="s">
         <v>207</v>
       </c>
-      <c r="F1042" t="s">
-        <v>113</v>
+      <c r="F1042" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1042" t="s">
         <v>8</v>
@@ -35136,8 +35206,10 @@
       <c r="E1043" t="s">
         <v>207</v>
       </c>
-      <c r="F1043" t="s">
-        <v>113</v>
+      <c r="F1043" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1043" t="s">
         <v>13</v>
@@ -35168,8 +35240,10 @@
       <c r="E1044" t="s">
         <v>207</v>
       </c>
-      <c r="F1044" t="s">
-        <v>113</v>
+      <c r="F1044" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1044" t="s">
         <v>10</v>
@@ -35200,8 +35274,10 @@
       <c r="E1045" t="s">
         <v>207</v>
       </c>
-      <c r="F1045" t="s">
-        <v>113</v>
+      <c r="F1045" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1045" t="s">
         <v>12</v>
@@ -35232,8 +35308,10 @@
       <c r="E1046" t="s">
         <v>207</v>
       </c>
-      <c r="F1046" t="s">
-        <v>113</v>
+      <c r="F1046" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1046" t="s">
         <v>33</v>
@@ -35264,8 +35342,10 @@
       <c r="E1047" t="s">
         <v>207</v>
       </c>
-      <c r="F1047" t="s">
-        <v>113</v>
+      <c r="F1047" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1047" t="s">
         <v>34</v>
@@ -46816,8 +46896,10 @@
       <c r="E1408" t="s">
         <v>207</v>
       </c>
-      <c r="F1408" t="s">
-        <v>113</v>
+      <c r="F1408" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1408" t="s">
         <v>32</v>
@@ -46848,8 +46930,10 @@
       <c r="E1409" t="s">
         <v>207</v>
       </c>
-      <c r="F1409" t="s">
-        <v>113</v>
+      <c r="F1409" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1409" t="s">
         <v>34</v>
@@ -46880,8 +46964,10 @@
       <c r="E1410" t="s">
         <v>207</v>
       </c>
-      <c r="F1410" t="s">
-        <v>113</v>
+      <c r="F1410" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1410" t="s">
         <v>35</v>
@@ -46912,8 +46998,10 @@
       <c r="E1411" t="s">
         <v>207</v>
       </c>
-      <c r="F1411" t="s">
-        <v>113</v>
+      <c r="F1411" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1411" t="s">
         <v>5</v>
@@ -46944,8 +47032,10 @@
       <c r="E1412" t="s">
         <v>207</v>
       </c>
-      <c r="F1412" t="s">
-        <v>113</v>
+      <c r="F1412" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1412" t="s">
         <v>2</v>
@@ -46976,8 +47066,10 @@
       <c r="E1413" t="s">
         <v>207</v>
       </c>
-      <c r="F1413" t="s">
-        <v>113</v>
+      <c r="F1413" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1413" t="s">
         <v>3</v>
@@ -47008,8 +47100,10 @@
       <c r="E1414" t="s">
         <v>207</v>
       </c>
-      <c r="F1414" t="s">
-        <v>113</v>
+      <c r="F1414" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1414" t="s">
         <v>6</v>
@@ -47040,8 +47134,10 @@
       <c r="E1415" t="s">
         <v>207</v>
       </c>
-      <c r="F1415" t="s">
-        <v>113</v>
+      <c r="F1415" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1415" t="s">
         <v>0</v>
@@ -47072,8 +47168,10 @@
       <c r="E1416" t="s">
         <v>207</v>
       </c>
-      <c r="F1416" t="s">
-        <v>113</v>
+      <c r="F1416" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1416" t="s">
         <v>4</v>
@@ -47104,8 +47202,10 @@
       <c r="E1417" t="s">
         <v>207</v>
       </c>
-      <c r="F1417" t="s">
-        <v>113</v>
+      <c r="F1417" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1417" t="s">
         <v>33</v>
@@ -47136,8 +47236,10 @@
       <c r="E1418" t="s">
         <v>207</v>
       </c>
-      <c r="F1418" t="s">
-        <v>113</v>
+      <c r="F1418" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1418" t="s">
         <v>7</v>
@@ -47168,8 +47270,10 @@
       <c r="E1419" t="s">
         <v>207</v>
       </c>
-      <c r="F1419" t="s">
-        <v>113</v>
+      <c r="F1419" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1419" t="s">
         <v>12</v>
@@ -47200,8 +47304,10 @@
       <c r="E1420" t="s">
         <v>207</v>
       </c>
-      <c r="F1420" t="s">
-        <v>113</v>
+      <c r="F1420" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1420" t="s">
         <v>11</v>
@@ -47232,8 +47338,10 @@
       <c r="E1421" t="s">
         <v>207</v>
       </c>
-      <c r="F1421" t="s">
-        <v>113</v>
+      <c r="F1421" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1421" t="s">
         <v>9</v>
@@ -47264,8 +47372,10 @@
       <c r="E1422" t="s">
         <v>207</v>
       </c>
-      <c r="F1422" t="s">
-        <v>113</v>
+      <c r="F1422" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1422" t="s">
         <v>13</v>
@@ -47296,8 +47406,10 @@
       <c r="E1423" t="s">
         <v>207</v>
       </c>
-      <c r="F1423" t="s">
-        <v>113</v>
+      <c r="F1423" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1423" t="s">
         <v>14</v>
@@ -47328,8 +47440,10 @@
       <c r="E1424" t="s">
         <v>207</v>
       </c>
-      <c r="F1424" t="s">
-        <v>113</v>
+      <c r="F1424" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1424" t="s">
         <v>36</v>
@@ -47360,8 +47474,10 @@
       <c r="E1425" t="s">
         <v>207</v>
       </c>
-      <c r="F1425" t="s">
-        <v>113</v>
+      <c r="F1425" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1425" t="s">
         <v>1</v>
@@ -47392,8 +47508,10 @@
       <c r="E1426" t="s">
         <v>207</v>
       </c>
-      <c r="F1426" t="s">
-        <v>113</v>
+      <c r="F1426" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1426" t="s">
         <v>10</v>
@@ -47424,8 +47542,10 @@
       <c r="E1427" t="s">
         <v>207</v>
       </c>
-      <c r="F1427" t="s">
-        <v>113</v>
+      <c r="F1427" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="G1427" t="s">
         <v>8</v>
@@ -85869,8 +85989,10 @@
       <c r="C9" s="8">
         <v>46074</v>
       </c>
-      <c r="D9" t="s">
-        <v>113</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="E9" t="str">
         <f t="shared" si="2"/>
@@ -86375,8 +86497,10 @@
       <c r="C26" s="8">
         <v>46278</v>
       </c>
-      <c r="D26" s="6" t="s">
-        <v>113</v>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="E26" t="str">
         <f t="shared" ref="E26:E41" si="5">VLOOKUP(D26,$K$1:$L$43,2,FALSE)</f>
@@ -86481,8 +86605,10 @@
       <c r="G29" s="11">
         <v>0.25</v>
       </c>
-      <c r="K29" t="s">
-        <v>113</v>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
       </c>
       <c r="L29" t="s">
         <v>157</v>
@@ -86636,8 +86762,10 @@
       <c r="G34" s="11">
         <v>0.25</v>
       </c>
-      <c r="K34" t="s">
-        <v>204</v>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Spanish GP</t>
+        </is>
       </c>
       <c r="L34" t="s">
         <v>203</v>
@@ -86804,8 +86932,10 @@
       <c r="C41" s="8">
         <v>46383</v>
       </c>
-      <c r="D41" t="s">
-        <v>204</v>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Spanish GP</t>
+        </is>
       </c>
       <c r="E41" t="str">
         <f t="shared" si="5"/>

</xml_diff>

<commit_message>
Import R results: Barcelona-Catalunya GP (round 6)
</commit_message>
<xml_diff>
--- a/F1_Standings.xlsx
+++ b/F1_Standings.xlsx
@@ -61953,179 +61953,1235 @@
       </c>
     </row>
     <row r="1802" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="F1802" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1802" t="s">
-        <v>37</v>
+      <c r="A1802" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1802" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1802" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1802">
+        <v>6</v>
+      </c>
+      <c r="E1802" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1802" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1802" t="inlineStr">
+        <is>
+          <t>TomasRodri21</t>
+        </is>
+      </c>
+      <c r="H1802" t="inlineStr">
+        <is>
+          <t>McLaren</t>
+        </is>
+      </c>
+      <c r="I1802">
+        <v>1</v>
+      </c>
+      <c r="J1802">
+        <v>25</v>
+      </c>
+      <c r="K1802" t="inlineStr">
+        <is>
+          <t>90:46.401</t>
+        </is>
+      </c>
+      <c r="L1802" t="inlineStr">
+        <is>
+          <t>1:18.091</t>
+        </is>
       </c>
     </row>
     <row r="1803" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="F1803" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1803" t="s">
-        <v>37</v>
+      <c r="A1803" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1803" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1803" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1803">
+        <v>6</v>
+      </c>
+      <c r="E1803" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1803" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1803" t="inlineStr">
+        <is>
+          <t>Polingua</t>
+        </is>
+      </c>
+      <c r="H1803" t="inlineStr">
+        <is>
+          <t>Red Bull</t>
+        </is>
+      </c>
+      <c r="I1803">
+        <v>2</v>
+      </c>
+      <c r="J1803">
+        <v>18</v>
+      </c>
+      <c r="K1803" t="inlineStr">
+        <is>
+          <t>+28.697</t>
+        </is>
+      </c>
+      <c r="L1803" t="inlineStr">
+        <is>
+          <t>1:17.311</t>
+        </is>
       </c>
     </row>
     <row r="1804" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="F1804" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1804" t="s">
-        <v>37</v>
+      <c r="A1804" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1804" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1804" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1804">
+        <v>6</v>
+      </c>
+      <c r="E1804" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1804" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1804" t="inlineStr">
+        <is>
+          <t>Charles Leclerc</t>
+        </is>
+      </c>
+      <c r="H1804" t="inlineStr">
+        <is>
+          <t>Ferrari</t>
+        </is>
+      </c>
+      <c r="I1804">
+        <v>3</v>
+      </c>
+      <c r="J1804">
+        <v>15</v>
+      </c>
+      <c r="K1804" t="inlineStr">
+        <is>
+          <t>+29.749</t>
+        </is>
+      </c>
+      <c r="L1804" t="inlineStr">
+        <is>
+          <t>1:19.163</t>
+        </is>
       </c>
     </row>
     <row r="1805" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="F1805" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1805" t="s">
-        <v>37</v>
+      <c r="A1805" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1805" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1805" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1805">
+        <v>6</v>
+      </c>
+      <c r="E1805" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1805" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1805" t="inlineStr">
+        <is>
+          <t>Kimi Antonelli</t>
+        </is>
+      </c>
+      <c r="H1805" t="inlineStr">
+        <is>
+          <t>Mercedes</t>
+        </is>
+      </c>
+      <c r="I1805">
+        <v>4</v>
+      </c>
+      <c r="J1805">
+        <v>12</v>
+      </c>
+      <c r="K1805" t="inlineStr">
+        <is>
+          <t>+30.216</t>
+        </is>
+      </c>
+      <c r="L1805" t="inlineStr">
+        <is>
+          <t>1:19.234</t>
+        </is>
       </c>
     </row>
     <row r="1806" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="F1806" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1806" t="s">
-        <v>37</v>
+      <c r="A1806" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1806" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1806" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1806">
+        <v>6</v>
+      </c>
+      <c r="E1806" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1806" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1806" t="inlineStr">
+        <is>
+          <t>Lewis Hamilton</t>
+        </is>
+      </c>
+      <c r="H1806" t="inlineStr">
+        <is>
+          <t>Ferrari</t>
+        </is>
+      </c>
+      <c r="I1806">
+        <v>5</v>
+      </c>
+      <c r="J1806">
+        <v>10</v>
+      </c>
+      <c r="K1806" t="inlineStr">
+        <is>
+          <t>+33.751</t>
+        </is>
+      </c>
+      <c r="L1806" t="inlineStr">
+        <is>
+          <t>1:19.064</t>
+        </is>
       </c>
     </row>
     <row r="1807" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="F1807" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1807" t="s">
-        <v>37</v>
+      <c r="A1807" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1807" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1807" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1807">
+        <v>6</v>
+      </c>
+      <c r="E1807" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1807" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1807" t="inlineStr">
+        <is>
+          <t>Max Verstappen</t>
+        </is>
+      </c>
+      <c r="H1807" t="inlineStr">
+        <is>
+          <t>Red Bull</t>
+        </is>
+      </c>
+      <c r="I1807">
+        <v>6</v>
+      </c>
+      <c r="J1807">
+        <v>8</v>
+      </c>
+      <c r="K1807" t="inlineStr">
+        <is>
+          <t>+39.225</t>
+        </is>
+      </c>
+      <c r="L1807" t="inlineStr">
+        <is>
+          <t>1:19.240</t>
+        </is>
       </c>
     </row>
     <row r="1808" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="F1808" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1808" t="s">
-        <v>37</v>
+      <c r="A1808" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1808" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1808" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1808">
+        <v>6</v>
+      </c>
+      <c r="E1808" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1808" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1808" t="inlineStr">
+        <is>
+          <t>Carlos Sainz Jr.</t>
+        </is>
+      </c>
+      <c r="H1808" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="I1808">
+        <v>7</v>
+      </c>
+      <c r="J1808">
+        <v>6</v>
+      </c>
+      <c r="K1808" t="inlineStr">
+        <is>
+          <t>+58.210</t>
+        </is>
+      </c>
+      <c r="L1808" t="inlineStr">
+        <is>
+          <t>1:19.987</t>
+        </is>
       </c>
     </row>
     <row r="1809" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1809" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1809" t="s">
-        <v>37</v>
+      <c r="A1809" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1809" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1809" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1809">
+        <v>6</v>
+      </c>
+      <c r="E1809" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1809" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1809" t="inlineStr">
+        <is>
+          <t>Alexander Albon</t>
+        </is>
+      </c>
+      <c r="H1809" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="I1809">
+        <v>8</v>
+      </c>
+      <c r="J1809">
+        <v>4</v>
+      </c>
+      <c r="K1809" t="inlineStr">
+        <is>
+          <t>+1:00.187</t>
+        </is>
+      </c>
+      <c r="L1809" t="inlineStr">
+        <is>
+          <t>1:19.975</t>
+        </is>
       </c>
     </row>
     <row r="1810" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1810" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1810" t="s">
-        <v>37</v>
+      <c r="A1810" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1810" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1810" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1810">
+        <v>6</v>
+      </c>
+      <c r="E1810" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1810" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1810" t="inlineStr">
+        <is>
+          <t>Pierre Gasly</t>
+        </is>
+      </c>
+      <c r="H1810" t="inlineStr">
+        <is>
+          <t>Alpine</t>
+        </is>
+      </c>
+      <c r="I1810">
+        <v>9</v>
+      </c>
+      <c r="J1810">
+        <v>2</v>
+      </c>
+      <c r="K1810" t="inlineStr">
+        <is>
+          <t>+1:13.080</t>
+        </is>
+      </c>
+      <c r="L1810" t="inlineStr">
+        <is>
+          <t>1:20.055</t>
+        </is>
       </c>
     </row>
     <row r="1811" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1811" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1811" t="s">
-        <v>37</v>
+      <c r="A1811" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1811" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1811" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1811">
+        <v>6</v>
+      </c>
+      <c r="E1811" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1811" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1811" t="inlineStr">
+        <is>
+          <t>Arvid Lidblad</t>
+        </is>
+      </c>
+      <c r="H1811" t="inlineStr">
+        <is>
+          <t>Racing Bulls</t>
+        </is>
+      </c>
+      <c r="I1811">
+        <v>10</v>
+      </c>
+      <c r="J1811">
+        <v>1</v>
+      </c>
+      <c r="K1811" t="inlineStr">
+        <is>
+          <t>+1:13.676</t>
+        </is>
+      </c>
+      <c r="L1811" t="inlineStr">
+        <is>
+          <t>1:20.558</t>
+        </is>
       </c>
     </row>
     <row r="1812" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1812" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1812" t="s">
-        <v>37</v>
+      <c r="A1812" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1812" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1812" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1812">
+        <v>6</v>
+      </c>
+      <c r="E1812" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1812" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1812" t="inlineStr">
+        <is>
+          <t>Franco Colapinto</t>
+        </is>
+      </c>
+      <c r="H1812" t="inlineStr">
+        <is>
+          <t>Alpine</t>
+        </is>
+      </c>
+      <c r="I1812">
+        <v>11</v>
+      </c>
+      <c r="J1812">
+        <v>0</v>
+      </c>
+      <c r="K1812" t="inlineStr">
+        <is>
+          <t>+1:21.947</t>
+        </is>
+      </c>
+      <c r="L1812" t="inlineStr">
+        <is>
+          <t>1:20.411</t>
+        </is>
       </c>
     </row>
     <row r="1813" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1813" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1813" t="s">
-        <v>37</v>
+      <c r="A1813" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1813" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1813" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1813">
+        <v>6</v>
+      </c>
+      <c r="E1813" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1813" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1813" t="inlineStr">
+        <is>
+          <t>Fernando Alonso</t>
+        </is>
+      </c>
+      <c r="H1813" t="inlineStr">
+        <is>
+          <t>Aston Martin</t>
+        </is>
+      </c>
+      <c r="I1813">
+        <v>12</v>
+      </c>
+      <c r="J1813">
+        <v>0</v>
+      </c>
+      <c r="K1813" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1813" t="inlineStr">
+        <is>
+          <t>1:20.130</t>
+        </is>
       </c>
     </row>
     <row r="1814" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1814" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1814" t="s">
-        <v>37</v>
+      <c r="A1814" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1814" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1814" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1814">
+        <v>6</v>
+      </c>
+      <c r="E1814" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1814" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1814" t="inlineStr">
+        <is>
+          <t>Nico Hülkenberg</t>
+        </is>
+      </c>
+      <c r="H1814" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="I1814">
+        <v>13</v>
+      </c>
+      <c r="J1814">
+        <v>0</v>
+      </c>
+      <c r="K1814" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1814" t="inlineStr">
+        <is>
+          <t>1:20.555</t>
+        </is>
       </c>
     </row>
     <row r="1815" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1815" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1815" t="s">
-        <v>37</v>
+      <c r="A1815" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1815" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1815" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1815">
+        <v>6</v>
+      </c>
+      <c r="E1815" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1815" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1815" t="inlineStr">
+        <is>
+          <t>Sergio Perez</t>
+        </is>
+      </c>
+      <c r="H1815" t="inlineStr">
+        <is>
+          <t>Cadillac</t>
+        </is>
+      </c>
+      <c r="I1815">
+        <v>14</v>
+      </c>
+      <c r="J1815">
+        <v>0</v>
+      </c>
+      <c r="K1815" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1815" t="inlineStr">
+        <is>
+          <t>1:20.831</t>
+        </is>
       </c>
     </row>
     <row r="1816" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1816" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1816" t="s">
-        <v>37</v>
+      <c r="A1816" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1816" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1816" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1816">
+        <v>6</v>
+      </c>
+      <c r="E1816" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1816" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1816" t="inlineStr">
+        <is>
+          <t>Lance Stroll</t>
+        </is>
+      </c>
+      <c r="H1816" t="inlineStr">
+        <is>
+          <t>Aston Martin</t>
+        </is>
+      </c>
+      <c r="I1816">
+        <v>15</v>
+      </c>
+      <c r="J1816">
+        <v>0</v>
+      </c>
+      <c r="K1816" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1816" t="inlineStr">
+        <is>
+          <t>1:21.203</t>
+        </is>
       </c>
     </row>
     <row r="1817" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1817" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1817" t="s">
-        <v>37</v>
+      <c r="A1817" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1817" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1817" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1817">
+        <v>6</v>
+      </c>
+      <c r="E1817" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1817" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1817" t="inlineStr">
+        <is>
+          <t>Oliver Bearman</t>
+        </is>
+      </c>
+      <c r="H1817" t="inlineStr">
+        <is>
+          <t>Haas</t>
+        </is>
+      </c>
+      <c r="I1817">
+        <v>16</v>
+      </c>
+      <c r="J1817">
+        <v>0</v>
+      </c>
+      <c r="K1817" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1817" t="inlineStr">
+        <is>
+          <t>1:20.637</t>
+        </is>
       </c>
     </row>
     <row r="1818" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1818" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1818" t="s">
-        <v>37</v>
+      <c r="A1818" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1818" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1818" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1818">
+        <v>6</v>
+      </c>
+      <c r="E1818" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1818" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1818" t="inlineStr">
+        <is>
+          <t>Esteban Ocon</t>
+        </is>
+      </c>
+      <c r="H1818" t="inlineStr">
+        <is>
+          <t>Haas</t>
+        </is>
+      </c>
+      <c r="I1818">
+        <v>17</v>
+      </c>
+      <c r="J1818">
+        <v>0</v>
+      </c>
+      <c r="K1818" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1818" t="inlineStr">
+        <is>
+          <t>1:21.392</t>
+        </is>
       </c>
     </row>
     <row r="1819" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1819" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1819" t="s">
-        <v>37</v>
+      <c r="A1819" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1819" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1819" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1819">
+        <v>6</v>
+      </c>
+      <c r="E1819" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1819" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1819" t="inlineStr">
+        <is>
+          <t>Valtteri Bottas</t>
+        </is>
+      </c>
+      <c r="H1819" t="inlineStr">
+        <is>
+          <t>Cadillac</t>
+        </is>
+      </c>
+      <c r="I1819">
+        <v>18</v>
+      </c>
+      <c r="J1819">
+        <v>0</v>
+      </c>
+      <c r="K1819" t="inlineStr">
+        <is>
+          <t>+2 Laps</t>
+        </is>
+      </c>
+      <c r="L1819" t="inlineStr">
+        <is>
+          <t>1:21.630</t>
+        </is>
       </c>
     </row>
     <row r="1820" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1820" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1820" t="s">
-        <v>37</v>
+      <c r="A1820" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1820" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1820" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1820">
+        <v>6</v>
+      </c>
+      <c r="E1820" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1820" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1820" t="inlineStr">
+        <is>
+          <t>Gabriel Bortoleto</t>
+        </is>
+      </c>
+      <c r="H1820" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="I1820">
+        <v>19</v>
+      </c>
+      <c r="J1820">
+        <v>0</v>
+      </c>
+      <c r="K1820" t="inlineStr">
+        <is>
+          <t>+2 Laps</t>
+        </is>
+      </c>
+      <c r="L1820" t="inlineStr">
+        <is>
+          <t>1:21.409</t>
+        </is>
       </c>
     </row>
     <row r="1821" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1821" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1821" t="s">
-        <v>37</v>
+      <c r="A1821" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1821" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1821" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1821">
+        <v>6</v>
+      </c>
+      <c r="E1821" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1821" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1821" t="inlineStr">
+        <is>
+          <t>Fatacuida</t>
+        </is>
+      </c>
+      <c r="H1821" t="inlineStr">
+        <is>
+          <t>Mercedes</t>
+        </is>
+      </c>
+      <c r="I1821">
+        <v>20</v>
+      </c>
+      <c r="J1821">
+        <v>0</v>
+      </c>
+      <c r="K1821" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="L1821" t="inlineStr">
+        <is>
+          <t>1:20.229</t>
+        </is>
       </c>
     </row>
     <row r="1822" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1822" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1822" t="s">
-        <v>37</v>
+      <c r="A1822" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1822" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1822" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1822">
+        <v>6</v>
+      </c>
+      <c r="E1822" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1822" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1822" t="inlineStr">
+        <is>
+          <t>Liam Lawson</t>
+        </is>
+      </c>
+      <c r="H1822" t="inlineStr">
+        <is>
+          <t>Racing Bulls</t>
+        </is>
+      </c>
+      <c r="I1822">
+        <v>21</v>
+      </c>
+      <c r="J1822">
+        <v>0</v>
+      </c>
+      <c r="K1822" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="L1822" t="inlineStr">
+        <is>
+          <t>1:20.825</t>
+        </is>
       </c>
     </row>
     <row r="1823" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1823" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1823" t="s">
-        <v>37</v>
+      <c r="A1823" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1823" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1823" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1823">
+        <v>6</v>
+      </c>
+      <c r="E1823" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1823" t="inlineStr">
+        <is>
+          <t>Barcelona-Catalunya GP</t>
+        </is>
+      </c>
+      <c r="G1823" t="inlineStr">
+        <is>
+          <t>Lando Norris</t>
+        </is>
+      </c>
+      <c r="H1823" t="inlineStr">
+        <is>
+          <t>McLaren</t>
+        </is>
+      </c>
+      <c r="I1823">
+        <v>22</v>
+      </c>
+      <c r="J1823">
+        <v>0</v>
+      </c>
+      <c r="K1823" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="L1823" t="inlineStr">
+        <is>
+          <t>1:19.683</t>
+        </is>
       </c>
     </row>
     <row r="1824" spans="6:10" x14ac:dyDescent="0.45">
@@ -86506,8 +87562,10 @@
         <f t="shared" ref="E26:E41" si="5">VLOOKUP(D26,$K$1:$L$43,2,FALSE)</f>
         <v>Circuit de Barcelona-Catalunya</v>
       </c>
-      <c r="F26" t="s">
-        <v>191</v>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
       </c>
       <c r="G26" s="11">
         <v>0.25</v>

</xml_diff>